<commit_message>
progress: 71 village workbooks (sivaramans-llin 2026-10-10T20:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Erukuvoy_13.348349_80.049903.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Erukuvoy_13.348349_80.049903.xlsx
@@ -866,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -873,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -880,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -887,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -894,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -901,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B1, 6B2, 6B3, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -908,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -915,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17A, 17B, 17C, 17D, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 3, 30, 31, 32, 33, 34A, 34B, 35, 36, 37, 4, 5, 6A, 6B, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -922,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F1, 1F2, 1F3, 1G, 1H, 1I, 1J, 2A, 2B, 2C, 2D, 2E, 2F1, 2F2, 2F3, 2G, 2H, 2I, 2J</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -929,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13A, 13B, 14, 15, 16, 1A, 1B, 1C, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -936,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 12A, 12B, 12C, 13A, 13B, 14, 15, 16, 17, 18, 19, 2, 20, 21, 3A, 3B, 3C, 4A, 4B1, 4B2A, 4B2B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -943,6 +998,11 @@
           <t>141A</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -950,6 +1010,11 @@
           <t>141B</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -957,6 +1022,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -964,6 +1034,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -971,6 +1046,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A, 1B1, 1B2, 2, 3A, 3B, 4A, 4B, 5A1, 5A2, 5B, 5C, 5D1, 5D2, 6A1, 6A2, 6A3, 6A4, 6A5A1, 6A5A2, 6A5B, 6A6A1, 6A6B, 6A6C, 6A6D, 6A6E, 6A6F, 6B1A1, 6B1B, 6B1C, 6B1D, 6B1E, 6B1F, 6B1G, 6B1H, 6B2, 7A1, 7A2A, 7A2B1A1, 7A2B2, 7A2B3, 7A2B4, 7A2B5, 7A3A, 7A3B, 7A3CA, 7A3CB, 7A3D, 7A3E, 7A4A1, 7A4A2, 7A4A3, 7A4B, 7B1A, 7B1B, 7B1C, 7B1D, 7B1E, 7B1F, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -978,6 +1058,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -985,6 +1070,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -992,6 +1082,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -999,6 +1094,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1006,6 +1106,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1013,6 +1118,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1020,6 +1130,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3A3, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1027,6 +1142,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1034,6 +1154,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1041,6 +1166,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1048,6 +1178,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1055,6 +1190,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B1C, 1B2A, 1B2B, 1C1, 1C2, 2A, 2B, 2C, 2D, 2E, 2F, 2G</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1062,6 +1202,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1069,6 +1214,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A1, 1A2A2, 1A2B, 1B1A, 1B1B, 1B2, 1B3, 1B4, 2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1076,6 +1226,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1083,6 +1238,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1090,6 +1250,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 18, 19, 2A, 2B, 3, 4, 5, 6A, 6B, 6C, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1097,6 +1262,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3A, 3B, 3C1, 3C2, 3C3, 3C4</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1104,6 +1274,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1, 1C2, 1C3, 1D1, 1D2, 1D3, 1E1, 1E2, 1E3, 1E4, 1E5, 1E6, 1F1, 1F2, 1F3, 1F4, 1F5, 2A, 2B, 3A1, 3A2, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1111,6 +1286,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F1, 1F2, 1F3, 2A, 2B1, 2B2, 2B3, 2C1, 2C2, 2C3</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1118,6 +1298,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1125,11 +1310,21 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
           <t>17</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 73 village workbooks (sivaramans-llin 2026-10-10T22:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Erukuvoy_13.348349_80.049903.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Erukuvoy_13.348349_80.049903.xlsx
@@ -1334,6 +1334,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25A, 25B, 26, 27, 28, 29, 3, 30A, 30B, 30C, 31, 32, 33A, 33B, 34, 35, 36, 37, 38A, 38B, 4A, 4B, 5A, 5B, 5C, 5D1, 5D2, 5E, 5F, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1341,6 +1346,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1348,6 +1358,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1355,6 +1370,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11A1, 11A2, 11A3, 11B, 12A, 12B, 12C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1362,6 +1382,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1369,6 +1394,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1376,6 +1406,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1383,6 +1418,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1390,6 +1430,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1397,6 +1442,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1404,6 +1454,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1411,6 +1466,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1418,6 +1478,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1425,6 +1490,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1432,6 +1502,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1439,6 +1514,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1446,6 +1526,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1453,6 +1538,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1460,6 +1550,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1467,6 +1562,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1474,6 +1574,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1481,11 +1586,21 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
           <t>38</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 74 village workbooks (sivaramans-llin 2026-10-10T22:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Erukuvoy_13.348349_80.049903.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Erukuvoy_13.348349_80.049903.xlsx
@@ -1610,6 +1610,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1617,6 +1622,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1624,6 +1634,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1631,6 +1646,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1638,6 +1658,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1645,6 +1670,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1652,6 +1682,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2A, 2B, 3A1A, 3A1B, 3A2, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1659,6 +1694,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1666,6 +1706,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6A, 6B, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1673,6 +1718,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1680,6 +1730,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3, 4A, 4B, 5, 6, 7, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1687,6 +1742,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1694,6 +1754,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1701,6 +1766,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1708,6 +1778,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1715,6 +1790,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1722,6 +1802,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1729,6 +1814,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1736,6 +1826,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1743,6 +1838,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1750,6 +1850,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1757,6 +1862,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1764,6 +1874,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2A, 3</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1771,6 +1886,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D1, 1D2, 1E, 1F, 1G, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1778,6 +1898,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1785,6 +1910,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1792,6 +1922,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1799,6 +1934,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1806,6 +1946,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1813,6 +1958,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1820,6 +1970,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1827,6 +1982,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1834,6 +1994,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B1, 12B2, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1841,6 +2006,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1848,6 +2018,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A1, 2A2, 2A3, 2A4, 2B, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1855,6 +2030,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1862,6 +2042,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1869,6 +2054,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B, 3, 4, 5A, 5B, 5C, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1876,6 +2066,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6A, 6B, 7, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1883,6 +2078,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13A1, 13A2, 13A3, 13B, 13C1, 13C2A, 13C2B, 13C3, 13D, 13E, 13F, 13G, 13H, 13I, 13J, 13K1, 13K2, 1A1, 1A2, 1B, 2A, 2B, 2C, 3, 4, 5A, 5B, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1890,6 +2090,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1897,6 +2102,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1904,6 +2114,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7A1, 7A2, 7B1, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1911,6 +2126,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1918,6 +2138,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1925,6 +2150,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1932,6 +2162,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1939,6 +2174,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1946,6 +2186,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1953,6 +2198,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1960,6 +2210,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1967,6 +2222,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1974,6 +2234,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1981,6 +2246,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1988,6 +2258,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -1995,6 +2270,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2002,6 +2282,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 2-10</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2009,6 +2294,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2016,6 +2306,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2023,6 +2318,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 1C, 1D, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2030,6 +2330,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2037,6 +2342,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 3</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2044,6 +2354,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2051,6 +2366,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2058,6 +2378,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1, 1C2, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B1, 6B2, 6B3, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2065,11 +2390,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1A1A1, 2B1A2, 2B1B, 2B2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1C3, 2A, 2B, 3A1A, 3A1B, 3A2, 3B, 4A1A1, 4A1B, 4A2, 4B, 4C</t>
         </is>
       </c>
     </row>

</xml_diff>